<commit_message>
updated eq id structure and auditing
</commit_message>
<xml_diff>
--- a/docs/scientific/quarto-scidoc/quarto_reference_audit.xlsx
+++ b/docs/scientific/quarto-scidoc/quarto_reference_audit.xlsx
@@ -26,27 +26,39 @@
     <sheet name="anchor_links" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="other_links" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="broken_internal_links" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="broken_internal_links1" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="equations" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="missing_eq_custom_ids" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="equation_id_mismatches" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="dup_eq_custom_ids" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="dup_eq_custom_groups" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'summary'!$A$1:$B$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'all_labels'!$A$1:$F$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'all_label_refs'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'duplicate_labels'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'duplicate_label_groups'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'summary'!$A$1:$B$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'all_labels'!$A$1:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'all_label_refs'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'duplicate_labels'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'duplicate_label_groups'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'missing_label_refs'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'unused_labels'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'unused_labels'!$A$1:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'bib_entries'!$A$1:$E$300</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bib_citations'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'bib_citations'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'duplicate_bib_keys'!$A$1:$F$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'duplicate_bib_groups'!$A$1:$C$70</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'missing_bib_cites'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'missing_bib_cites'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'missing_bib_files'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'hyperlinks'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'hyperlinks'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'external_links'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'internal_links'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'internal_links'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'anchor_links'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'other_links'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'broken_internal_links'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'broken_internal_links1'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'equations'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'missing_eq_custom_ids'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'equation_id_mismatches'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'dup_eq_custom_ids'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'dup_eq_custom_groups'!$A$1:$C$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,10 +467,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -482,7 +494,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C:\Users\gmg228\Documents\RuFaS\RuFaS\docs\scientific\quarto-test</t>
+          <t>C:\Users\gmg228\Documents\RuFaS\RuFaS\docs\scientific\quarto-scidoc</t>
         </is>
       </c>
     </row>
@@ -513,7 +525,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -523,7 +535,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +545,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -543,7 +555,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -563,7 +575,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -583,7 +595,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -613,7 +625,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -633,7 +645,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -653,7 +665,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -694,12 +706,62 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C:\Users\gmg228\Documents\RuFaS\RuFaS\docs\scientific\quarto-test\quarto_reference_audit.xlsx</t>
-        </is>
+          <t>C:\Users\gmg228\Documents\RuFaS\RuFaS\docs\scientific\quarto-scidoc\quarto_reference_audit.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>equations_found</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>missing_equation_custom_ids</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>equation_id_mismatches</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>duplicate_equation_custom_rows</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>duplicate_equation_custom_groups</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B23"/>
+  <autoFilter ref="A1:B28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10209,13 +10271,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10240,48 +10302,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>eqn-an-nrc-2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>animal.qmd</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>53</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>see @eqn-an-nrc-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>eqn-an-nrc-2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>equations.qmd</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>39</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>see @eqn-an-nrc-2</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10323,13 +10345,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="73" customWidth="1" min="6" max="6"/>
   </cols>
@@ -10397,10 +10419,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Animal module icon</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>resources/manure.png</t>
+          <t>resources/animal.png</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10410,15 +10436,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>manure.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>![](resources/manure.png){width=140px}</t>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
         </is>
       </c>
     </row>
@@ -10440,11 +10466,11 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>![](resources/manure.png){width=50%}</t>
+          <t>![](resources/manure.png){width=140px}</t>
         </is>
       </c>
     </row>
@@ -10452,60 +10478,86 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
+          <t>resources/manure.png</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>internal-file</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>manure.qmd</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>![](resources/manure.png){width=50%}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>resources/rufas.png</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>internal-file</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>index.qmd</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E6" t="n">
         <v>3</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>![](resources/rufas.png){width=90}</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>energykey</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>equations.qmd</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>48</v>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>calculation, please refer to the [energykey](energy requirements key).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10571,13 +10623,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="73" customWidth="1" min="6" max="6"/>
   </cols>
@@ -10645,10 +10697,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Animal module icon</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>resources/manure.png</t>
+          <t>resources/animal.png</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10658,15 +10714,15 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>manure.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>![](resources/manure.png){width=140px}</t>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
         </is>
       </c>
     </row>
@@ -10688,11 +10744,11 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>![](resources/manure.png){width=50%}</t>
+          <t>![](resources/manure.png){width=140px}</t>
         </is>
       </c>
     </row>
@@ -10700,30 +10756,56 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
+          <t>resources/manure.png</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>internal-file</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>manure.qmd</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>![](resources/manure.png){width=50%}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>resources/rufas.png</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>internal-file</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>index.qmd</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E6" t="n">
         <v>3</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>![](resources/rufas.png){width=90}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10795,7 +10877,7 @@
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="72" customWidth="1" min="6" max="6"/>
   </cols>
@@ -10850,11 +10932,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10929,15 +11011,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="73" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10975,7 +11057,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eq-energy</t>
+          <t>eq-an-nrc-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10985,11 +11067,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -10998,14 +11080,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>$$ {#eq-energy}</t>
+          <t>$$ {#eq-an-nrc-1}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>eq-nrc-cbw</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -11015,11 +11097,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -11028,14 +11110,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>$$CBW = MW * 0.06275$$ {#eq-nrc-cbw}</t>
+          <t>$$ {#eq-an-nrc-2}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>eq-nrc-cw</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -11045,11 +11127,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -11058,14 +11140,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>$$ CW = {(18 + (DOP - 190) * 0.665) * (\frac{CBW}{45}),\text{if}DOP &gt; 190.0} $$ {#eq-nrc-cw}</t>
+          <t>$$ {#eq-an-nrc-2}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>eq-nrc-ne-maint</t>
+          <t>eq-an-nrc-2-tagged</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -11075,11 +11157,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -11088,14 +11170,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>$$ NEmaint = 0.08 \times (BW - CW)^{0.75} $$ {#eq-nrc-ne-maint}</t>
+          <t>$$ {#eq-an-nrc-2-tagged}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>eq-nutrient-proportion</t>
+          <t>eq-an-nrc-3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -11105,11 +11187,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -11118,19 +11200,19 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>$$ {#eq-nutrient-proportion}</t>
+          <t>$$ {#eq-an-nrc-3}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fig-animal-icon</t>
+          <t>eq-an-nrc-4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Figure</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -11139,7 +11221,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -11148,19 +11230,19 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
+          <t>$$ {#eq-an-nrc-4}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-1</t>
+          <t>eq-an-nrc-5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -11169,7 +11251,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -11178,19 +11260,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-1}</t>
+          <t>$$ {#eq-an-nrc-5}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -11199,7 +11281,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -11208,28 +11290,28 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -11238,28 +11320,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-energy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -11268,28 +11350,28 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-energy}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-3</t>
+          <t>eq-nrc-cbw</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -11298,28 +11380,28 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-3}</t>
+          <t>$$ {#eq-nrc-cbw}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-4</t>
+          <t>eq-nrc-cbw-times</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -11328,28 +11410,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-4}</t>
+          <t>$$ {#eq-nrc-cbw-times}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-5</t>
+          <t>eq-nrc-cw</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -11358,28 +11440,28 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-5}</t>
+          <t>$$ {#eq-nrc-cw}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sec-nrc</t>
+          <t>eq-nrc-ne-maint</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -11388,28 +11470,28 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>## Nutrient Requirements of Dairy Cattle (NRC) {#sec-nrc}</t>
+          <t>$$ {#eq-nrc-ne-maint}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tbl-animal-inputs</t>
+          <t>eq-nutrient-proportion</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -11418,42 +11500,1595 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+          <t>$$ {#eq-nutrient-proportion}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>fig-animal-icon</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fig-animal-icon</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sec-nrc</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>45</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>## Nutrient Requirements of Dairy Cattle (NRC) {#sec-nrc}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>tbl-animal-inputs</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>18</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>25</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>manure.qmd</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D22" t="n">
         <v>26</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>attribute-id</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>: Example animal inputs {#tbl-animal-inputs}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>link_text</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>resolved_path</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>eq_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>custom_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>expected_custom_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>matches_expected</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>has_custom_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>equation_body</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.2)}</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AN.NRC.3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AN.NRC.3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.3)}</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AN.NRC.4</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AN.NRC.4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.4)}</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AN.NRC.5</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AN.NRC.5</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>34</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.5)}</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AN.NRC.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AN.NRC.1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>38</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.1)}</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.6)}</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>29</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.2)}</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>33</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.6)}</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>eq-nrc-cbw</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NRC.CBW</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>54</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>eq-nrc-cw</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NRC.CW</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>58</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>CW = {(18 + (DOP - 190) * 0.665) * \left(\frac{CBW}{45}\right), \text{if } DOP &gt; 190.0}</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>eq-nrc-ne-maint</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NRC.NE.MAINT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>64</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NEmaint = 0.08 \times (BW - CW)^{0.75}</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>eq-nrc-cbw-times</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NRC.CBW.TIMES</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>73</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>CBW = MW \times 0.06275</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2-tagged</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>AN.NRC.2.TAGGED</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>84</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \tag{AN.NRC.2}</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>eq-energy</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>94</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>E = mc^2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>eq-nutrient-proportion</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NUTRIENT.PROPORTION</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>\text{nutrient\_proportion\_to\_be\_removed} = \min\left( \frac{\text{mass\_requested\_nutrient}}{\text{manure\_nutrient\_available}}, 1 \right)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>eq_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>expected_custom_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>equation_body</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>eq-nrc-cbw</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NRC.CBW</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>54</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>eq-nrc-cw</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NRC.CW</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>58</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CW = {(18 + (DOP - 190) * 0.665) * \left(\frac{CBW}{45}\right), \text{if } DOP &gt; 190.0}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eq-nrc-ne-maint</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NRC.NE.MAINT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>64</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NEmaint = 0.08 \times (BW - CW)^{0.75}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>eq-nrc-cbw-times</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NRC.CBW.TIMES</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>73</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CBW = MW \times 0.06275</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eq-energy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>94</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>E = mc^2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>eq-nutrient-proportion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NUTRIENT.PROPORTION</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>\text{nutrient\_proportion\_to\_be\_removed} = \min\left( \frac{\text{mass\_requested\_nutrient}}{\text{manure\_nutrient\_available}}, 1 \right)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>eq_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>custom_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>expected_custom_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>equation_body</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2-tagged</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2.TAGGED</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>84</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \tag{AN.NRC.2}</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>custom_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>eq_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>equation_body</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.2)}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.2)}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2-tagged</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>84</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \tag{AN.NRC.2}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-6</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>42</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.6)}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-6</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>33</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CBW = MW * 0.06275 \qquad \text{(AN.NRC.6)}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>custom_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>files</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AN.NRC.2</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>animal.qmd; example_structures.qmd</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AN.NRC.6</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>animal.qmd; example_structures.qmd</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11464,12 +13099,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="66" customWidth="1" min="6" max="6"/>
@@ -11510,7 +13145,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eq-energy</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -11520,11 +13155,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -11533,42 +13168,132 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>See Equation @eq-energy.</t>
+          <t>See @eq-an-nrc-2.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>eq-an-nrc-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>37</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>@id</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>See @eq-an-nrc-2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eq-an-nrc-2-tagged</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>88</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>@id</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>See @eq-an-nrc-2-tagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>eq-energy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>98</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>@id</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>See Equation @eq-energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>eq-nrc-cbw</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Equation</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>equations.qmd</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>23</v>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>70</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>@id</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>@eq-nrc-cbw may be visually improved by using the `\times` LaTeX</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11579,15 +13304,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="73" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -11631,12 +13356,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -11645,7 +13370,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -11654,31 +13379,31 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-2}</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -11687,31 +13412,31 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-2}</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -11720,31 +13445,31 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tbl-animal-inputs</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -11753,7 +13478,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -11763,21 +13488,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tbl-animal-inputs</t>
+          <t>fig-animal-icon</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Figure</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>manure.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -11786,15 +13511,147 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fig-animal-icon</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>17</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>manure.qmd</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:G10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11805,13 +13662,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11839,32 +13696,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>animal.qmd; equations.qmd</t>
+          <t>animal.qmd; example_structures.qmd</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tbl-animal-inputs</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -11872,12 +13729,52 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>animal.qmd; manure.qmd</t>
+          <t>animal.qmd; example_structures.qmd</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fig-animal-icon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>animal.qmd; example_structures.qmd</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>animal.qmd; example_structures.qmd; manure.qmd</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11943,15 +13840,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="73" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11989,7 +13886,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eq-nrc-cw</t>
+          <t>eq-an-nrc-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -11999,11 +13896,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -12012,14 +13909,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>$$ CW = {(18 + (DOP - 190) * 0.665) * (\frac{CBW}{45}),\text{if}DOP &gt; 190.0} $$ {#eq-nrc-cw}</t>
+          <t>$$ {#eq-an-nrc-1}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>eq-nrc-ne-maint</t>
+          <t>eq-an-nrc-3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12029,11 +13926,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -12042,14 +13939,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>$$ NEmaint = 0.08 \times (BW - CW)^{0.75} $$ {#eq-nrc-ne-maint}</t>
+          <t>$$ {#eq-an-nrc-3}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>eq-nutrient-proportion</t>
+          <t>eq-an-nrc-4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12059,11 +13956,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>animal.qmd</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -12072,19 +13969,19 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>$$ {#eq-nutrient-proportion}</t>
+          <t>$$ {#eq-an-nrc-4}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-1</t>
+          <t>eq-an-nrc-5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -12093,7 +13990,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -12102,19 +13999,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-1}</t>
+          <t>$$ {#eq-an-nrc-5}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -12123,7 +14020,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -12132,28 +14029,28 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-an-nrc-6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -12162,28 +14059,28 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-an-nrc-6}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-2</t>
+          <t>eq-nrc-cbw-times</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -12192,28 +14089,28 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-2}</t>
+          <t>$$ {#eq-nrc-cbw-times}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-3</t>
+          <t>eq-nrc-cw</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -12222,28 +14119,28 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-3}</t>
+          <t>$$ {#eq-nrc-cw}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-4</t>
+          <t>eq-nrc-ne-maint</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -12252,28 +14149,28 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-4}</t>
+          <t>$$ {#eq-nrc-ne-maint}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>eqn-an-nrc-5</t>
+          <t>eq-nutrient-proportion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Equation</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>106</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -12282,7 +14179,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>:::{#eqn-an-nrc-5}</t>
+          <t>$$ {#eq-nutrient-proportion}</t>
         </is>
       </c>
     </row>
@@ -12319,21 +14216,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sec-nrc</t>
+          <t>fig-animal-icon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Figure</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>equations.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -12342,28 +14239,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>## Nutrient Requirements of Dairy Cattle (NRC) {#sec-nrc}</t>
+          <t>![Animal module icon](resources/animal.png){#fig-animal-icon width=35%}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tbl-animal-inputs</t>
+          <t>sec-nrc</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Table</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>animal.qmd</t>
+          <t>example_structures.qmd</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -12372,7 +14269,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+          <t>## Nutrient Requirements of Dairy Cattle (NRC) {#sec-nrc}</t>
         </is>
       </c>
     </row>
@@ -12389,25 +14286,85 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>animal.qmd</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>18</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>example_structures.qmd</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>25</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>attribute-id</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>: Example animal inputs {#tbl-animal-inputs}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tbl-animal-inputs</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>manure.qmd</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" t="n">
         <v>26</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>attribute-id</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>: Example animal inputs {#tbl-animal-inputs}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F15"/>
+  <autoFilter ref="A1:F17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19942,13 +21899,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19973,48 +21930,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>eqn-an-nrc-2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>animal.qmd</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>53</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>see @eqn-an-nrc-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>eqn-an-nrc-2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>equations.qmd</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>39</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>see @eqn-an-nrc-2</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>